<commit_message>
Assignment 1 automation setup
</commit_message>
<xml_diff>
--- a/it23214316_Test cases.xlsx
+++ b/it23214316_Test cases.xlsx
@@ -601,8 +601,16 @@
           <t>ළමයි disturb කරන්නේ නැතුව ඉන්න.</t>
         </is>
       </c>
-      <c r="E2" s="56" t="n"/>
-      <c r="F2" s="54" t="n"/>
+      <c r="E2" s="56" t="inlineStr">
+        <is>
+          <t>ළමයි disturb කරන්නේ නැතුව ඉන්න.</t>
+        </is>
+      </c>
+      <c r="F2" s="54" t="inlineStr">
+        <is>
+          <t>UI ERROR</t>
+        </is>
+      </c>
       <c r="G2" s="49" t="inlineStr">
         <is>
           <t>Question forms</t>
@@ -689,8 +697,12 @@
           <t>ඔයාට පුළුවන්ද මේ photo එක ආයෙත් එවන්න?</t>
         </is>
       </c>
-      <c r="E6" s="57" t="n"/>
-      <c r="F6" s="54" t="n"/>
+      <c r="E6" s="57" t="inlineStr"/>
+      <c r="F6" s="54" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="G6" s="49" t="inlineStr">
         <is>
           <t>Greetings</t>

</xml_diff>

<commit_message>
Fix Excel template (unmerge + 50 cases)
</commit_message>
<xml_diff>
--- a/it23214316_Test cases.xlsx
+++ b/it23214316_Test cases.xlsx
@@ -583,88 +583,122 @@
     <row r="2" ht="49.95000076293945" customHeight="1">
       <c r="A2" s="53" t="inlineStr">
         <is>
+          <t>Neg_0001</t>
+        </is>
+      </c>
+      <c r="B2" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C2" s="55" t="inlineStr">
+        <is>
+          <t>oyata dan kawadda enna puluwan?</t>
+        </is>
+      </c>
+      <c r="D2" s="56" t="inlineStr">
+        <is>
+          <t>ඔයාට දැන් කවද්ද එන්න පුළුවන්?</t>
+        </is>
+      </c>
+      <c r="E2" s="56" t="n"/>
+      <c r="F2" s="54" t="n"/>
+      <c r="G2" s="49" t="inlineStr">
+        <is>
+          <t>Question forms</t>
+        </is>
+      </c>
+      <c r="H2" s="49" t="inlineStr">
+        <is>
+          <t>Evidence: Question asking arrival time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="49.95000076293945" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Neg_0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>oya monawada hithanne me gana?</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ඔයා මොනවද හිතන්නේ මේ ගැන?</t>
+        </is>
+      </c>
+      <c r="G3" s="49" t="inlineStr">
+        <is>
+          <t>Question forms</t>
+        </is>
+      </c>
+      <c r="H3" s="49" t="inlineStr">
+        <is>
+          <t>Evidence: Question asking opinion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="49.95000076293945" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Neg_0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>wahama meka copy karala eyaata yawanna.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>වහාම මේක copy කරලා එයාට යවන්න.</t>
+        </is>
+      </c>
+      <c r="G4" s="49" t="inlineStr">
+        <is>
+          <t>Command forms</t>
+        </is>
+      </c>
+      <c r="H4" s="49" t="inlineStr">
+        <is>
+          <t>Evidence: Gives an instruction to send it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="49.95000076293945" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Neg_0004</t>
         </is>
       </c>
-      <c r="B2" s="54" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="C2" s="55" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>lamayi disturb karanne nathuwa inna.</t>
         </is>
       </c>
-      <c r="D2" s="56" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>ළමයි disturb කරන්නේ නැතුව ඉන්න.</t>
         </is>
       </c>
-      <c r="E2" s="56" t="inlineStr">
-        <is>
-          <t>ළමයි disturb කරන්නේ නැතුව ඉන්න.</t>
-        </is>
-      </c>
-      <c r="F2" s="54" t="inlineStr">
-        <is>
-          <t>UI ERROR</t>
-        </is>
-      </c>
-      <c r="G2" s="49" t="inlineStr">
-        <is>
-          <t>Question forms</t>
-        </is>
-      </c>
-      <c r="H2" s="49" t="inlineStr">
-        <is>
-          <t>Evidence: Question asking arrival time.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="49.95000076293945" customHeight="1">
-      <c r="A3" s="12" t="n"/>
-      <c r="B3" s="12" t="n"/>
-      <c r="C3" s="12" t="n"/>
-      <c r="D3" s="12" t="n"/>
-      <c r="E3" s="12" t="n"/>
-      <c r="F3" s="12" t="n"/>
-      <c r="G3" s="49" t="inlineStr">
-        <is>
-          <t>Question forms</t>
-        </is>
-      </c>
-      <c r="H3" s="49" t="inlineStr">
-        <is>
-          <t>Evidence: Question asking opinion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="49.95000076293945" customHeight="1">
-      <c r="A4" s="12" t="n"/>
-      <c r="B4" s="12" t="n"/>
-      <c r="C4" s="12" t="n"/>
-      <c r="D4" s="12" t="n"/>
-      <c r="E4" s="12" t="n"/>
-      <c r="F4" s="12" t="n"/>
-      <c r="G4" s="49" t="inlineStr">
-        <is>
-          <t>Command forms</t>
-        </is>
-      </c>
-      <c r="H4" s="49" t="inlineStr">
-        <is>
-          <t>Evidence: Gives an instruction to send it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="49.95000076293945" customHeight="1">
-      <c r="A5" s="13" t="n"/>
-      <c r="B5" s="13" t="n"/>
-      <c r="C5" s="13" t="n"/>
-      <c r="D5" s="13" t="n"/>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="13" t="n"/>
       <c r="G5" s="49" t="inlineStr">
         <is>
           <t>Command forms</t>
@@ -679,84 +713,122 @@
     <row r="6" ht="49.95000076293945" customHeight="1">
       <c r="A6" s="53" t="inlineStr">
         <is>
+          <t>Neg_0005</t>
+        </is>
+      </c>
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C6" s="55" t="inlineStr">
+        <is>
+          <t>suba dawasak! oya kohomada?</t>
+        </is>
+      </c>
+      <c r="D6" s="56" t="inlineStr">
+        <is>
+          <t>සුබ දවසක්! ඔයා කොහොමද?</t>
+        </is>
+      </c>
+      <c r="E6" s="57" t="n"/>
+      <c r="F6" s="54" t="n"/>
+      <c r="G6" s="49" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="H6" s="49" t="inlineStr">
+        <is>
+          <t>Evidence: Greeting + asking how they are.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="49.95000076293945" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Neg_0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>suba raththriyak wewa! hodata nidaganna.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>සුබ රාත්‍රියක් වේවා! හොඳට නිදාගන්න.</t>
+        </is>
+      </c>
+      <c r="G7" s="49" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="H7" s="49" t="inlineStr">
+        <is>
+          <t>Evidence: Good-night greeting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="49.95000076293945" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Neg_0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>karunakara mata poddak sahayogayak dennako.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>කරුණාකර මට පොඩ්ඩක් සහයෝගයක් දෙන්නකෝ.</t>
+        </is>
+      </c>
+      <c r="G8" s="49" t="inlineStr">
+        <is>
+          <t>Requests</t>
+        </is>
+      </c>
+      <c r="H8" s="49" t="inlineStr">
+        <is>
+          <t>Evidence: Polite request for help.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="49.95000076293945" customHeight="1">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Neg_0008</t>
         </is>
       </c>
-      <c r="B6" s="54" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="C6" s="55" t="inlineStr">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>oyata puluwanda me photo eka ayeth ewanna?</t>
         </is>
       </c>
-      <c r="D6" s="56" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>ඔයාට පුළුවන්ද මේ photo එක ආයෙත් එවන්න?</t>
         </is>
       </c>
-      <c r="E6" s="57" t="inlineStr"/>
-      <c r="F6" s="54" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="G6" s="49" t="inlineStr">
-        <is>
-          <t>Greetings</t>
-        </is>
-      </c>
-      <c r="H6" s="49" t="inlineStr">
-        <is>
-          <t>Evidence: Greeting + asking how they are.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="49.95000076293945" customHeight="1">
-      <c r="A7" s="12" t="n"/>
-      <c r="B7" s="12" t="n"/>
-      <c r="C7" s="12" t="n"/>
-      <c r="D7" s="12" t="n"/>
-      <c r="E7" s="12" t="n"/>
-      <c r="F7" s="12" t="n"/>
-      <c r="G7" s="49" t="inlineStr">
-        <is>
-          <t>Greetings</t>
-        </is>
-      </c>
-      <c r="H7" s="49" t="inlineStr">
-        <is>
-          <t>Evidence: Good-night greeting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="49.95000076293945" customHeight="1">
-      <c r="A8" s="12" t="n"/>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="49" t="inlineStr">
-        <is>
-          <t>Requests</t>
-        </is>
-      </c>
-      <c r="H8" s="49" t="inlineStr">
-        <is>
-          <t>Evidence: Polite request for help.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="49.95000076293945" customHeight="1">
-      <c r="A9" s="13" t="n"/>
-      <c r="B9" s="13" t="n"/>
-      <c r="C9" s="13" t="n"/>
-      <c r="D9" s="13" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n"/>
       <c r="G9" s="49" t="inlineStr">
         <is>
           <t>Requests</t>
@@ -2197,20 +2269,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="D6:D9"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="E6:E9"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="F6:F9"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C6:C9"/>
-    <mergeCell ref="D2:D5"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>